<commit_message>
Fixes und Erzeugung einer Debitor Nummer
</commit_message>
<xml_diff>
--- a/2026/Q2/26-11695.xlsx
+++ b/2026/Q2/26-11695.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://talkserv.sharepoint.com/sites/Verwaltung/Freigegebene Dokumente/General/Rechnungen/2026/Q2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Faktura3\2026\Q2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{822958D0-8872-44FF-A871-6249A72C4F9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C46D7C-D8A2-47E7-9BF2-D2170DE7BA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{8447C29A-FB4B-4CB6-8F32-1E303CFC6589}"/>
   </bookViews>
@@ -826,7 +826,7 @@
         <v>9</v>
       </c>
       <c r="D5" s="6">
-        <v>126630</v>
+        <v>12001</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -991,26 +991,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="51ef5d3b-d653-42a4-add8-264426d78878">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="c7246570-ebc5-4d46-bfb6-2bb15f49e607" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100CE022242B0FA754895983687E40C5944" ma:contentTypeVersion="13" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e0af8390dce88dec6c8e4268a89a0009">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="51ef5d3b-d653-42a4-add8-264426d78878" xmlns:ns3="c7246570-ebc5-4d46-bfb6-2bb15f49e607" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bfffb4cac3116553a071a02667a615cb" ns2:_="" ns3:_="">
     <xsd:import namespace="51ef5d3b-d653-42a4-add8-264426d78878"/>
@@ -1217,10 +1197,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="51ef5d3b-d653-42a4-add8-264426d78878">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="c7246570-ebc5-4d46-bfb6-2bb15f49e607" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE192174-18BA-48A7-A32D-2EC0F92514FD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C6C820-5FB0-4511-A528-6A834AA202C8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="51ef5d3b-d653-42a4-add8-264426d78878"/>
+    <ds:schemaRef ds:uri="c7246570-ebc5-4d46-bfb6-2bb15f49e607"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1237,20 +1248,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C6C820-5FB0-4511-A528-6A834AA202C8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE192174-18BA-48A7-A32D-2EC0F92514FD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="51ef5d3b-d653-42a4-add8-264426d78878"/>
-    <ds:schemaRef ds:uri="c7246570-ebc5-4d46-bfb6-2bb15f49e607"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>